<commit_message>
Auto: update Tushare CITIC data
</commit_message>
<xml_diff>
--- a/data/000985_prices.xlsx
+++ b/data/000985_prices.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2292"/>
+  <dimension ref="A1:G2293"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -53216,6 +53216,29 @@
       </c>
       <c r="G2292" t="inlineStr"/>
     </row>
+    <row r="2293">
+      <c r="A2293" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B2293" t="n">
+        <v>6113.17</v>
+      </c>
+      <c r="C2293" t="n">
+        <v>6232.53</v>
+      </c>
+      <c r="D2293" t="n">
+        <v>6061.39</v>
+      </c>
+      <c r="E2293" t="n">
+        <v>6119.24</v>
+      </c>
+      <c r="F2293" t="n">
+        <v>1397132253</v>
+      </c>
+      <c r="G2293" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Data: manual update through 2026-07-22
</commit_message>
<xml_diff>
--- a/data/000985_prices.xlsx
+++ b/data/000985_prices.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\gx_pit_mom_Auto_Bot\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06F272CE-DA5E-4931-93AB-58FF411B2C68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DB7CDDC-0E9B-4828-AA40-9E54D6259A1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3420" yWindow="3420" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -198,16 +198,16 @@
     <xf numFmtId="176" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -542,7 +542,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G2433"/>
+  <dimension ref="A1:G2436"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.36328125" bestFit="1" customWidth="1"/>
@@ -632,7 +632,7 @@
         <v>42570</v>
       </c>
       <c r="B7" s="7">
-        <f>[1]!WSD(B3,B6:G6,B1,B2,"unit=1","TradingCalendar=SSE","rptType=1","Version=1","ShowParams=Y","UnitMask=32","cols=6;rows=2427")</f>
+        <f>[1]!WSD(B3,B6:G6,B1,B2,"unit=1","TradingCalendar=SSE","rptType=1","Version=1","ShowParams=Y","UnitMask=32","cols=6;rows=2430")</f>
         <v>4799.9991</v>
       </c>
       <c r="C7" s="7">
@@ -56447,6 +56447,75 @@
       </c>
       <c r="G2433" s="7">
         <v>2602175889503</v>
+      </c>
+    </row>
+    <row r="2434" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2434" s="1">
+        <v>46223</v>
+      </c>
+      <c r="B2434" s="7">
+        <v>5731.2191000000003</v>
+      </c>
+      <c r="C2434" s="7">
+        <v>5772.2106999999996</v>
+      </c>
+      <c r="D2434" s="7">
+        <v>5539.0392000000002</v>
+      </c>
+      <c r="E2434" s="7">
+        <v>5638.6185999999998</v>
+      </c>
+      <c r="F2434" s="7">
+        <v>142987607433</v>
+      </c>
+      <c r="G2434" s="7">
+        <v>2650229559275</v>
+      </c>
+    </row>
+    <row r="2435" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2435" s="1">
+        <v>46224</v>
+      </c>
+      <c r="B2435" s="7">
+        <v>5663.8751000000002</v>
+      </c>
+      <c r="C2435" s="7">
+        <v>5834.1704</v>
+      </c>
+      <c r="D2435" s="7">
+        <v>5510.4002</v>
+      </c>
+      <c r="E2435" s="7">
+        <v>5833.7268000000004</v>
+      </c>
+      <c r="F2435" s="7">
+        <v>151541877453</v>
+      </c>
+      <c r="G2435" s="7">
+        <v>2901920156472</v>
+      </c>
+    </row>
+    <row r="2436" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2436" s="1">
+        <v>46225</v>
+      </c>
+      <c r="B2436" s="7">
+        <v>5792.4529000000002</v>
+      </c>
+      <c r="C2436" s="7">
+        <v>5871.8368</v>
+      </c>
+      <c r="D2436" s="7">
+        <v>5757.7520000000004</v>
+      </c>
+      <c r="E2436" s="7">
+        <v>5790.7622000000001</v>
+      </c>
+      <c r="F2436" s="7">
+        <v>125478979400</v>
+      </c>
+      <c r="G2436" s="7">
+        <v>2602930506546</v>
       </c>
     </row>
   </sheetData>

</xml_diff>